<commit_message>
feat(ak): import AK interim->real (scraped) + validate; 18th scraped state
AK 100-row SERFF scrape (189/189 in-target, 0 true misses) replaces AM Best interim.
New baseline: 18 states, raw 2947 / rolled 1826 / active@2026-06-11 550 / db md5
23f0bf29 (supersedes post-HI d3075558). Every delta == exactly AK (+100/+53/+23/+1);
17 prior scraped states byte-identical (import_gate_verify.py: ALL GATES PASS);
CA/NY/TX permanent intact. AK dropped from AMBEST_STATES, KEPT in COVERED_STATES;
validated:{true,true}; methodology 17->18. 8th interim->real point: value-agreement
41/41=100% on shared filings. COVERAGE-THIN finding corrected: AM Best undercounts
COUNTRY specifically (32 vs 2 — the enrichment, live Prospect signals); Liberty/
Farmers Form/Rule-only (AM Best 0 correct, not a gap). Recovered 2 material COUNTRY
CFPC (wrapped-name bug, B6 backlog MEDIUM).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Insurance Rate Data Scraper/output/ak_final_rates.xlsx
+++ b/Insurance Rate Data Scraper/output/ak_final_rates.xlsx
@@ -9454,7 +9454,7 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>2,162.300%</t>
+          <t>2162.300%</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
@@ -9549,7 +9549,7 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>2,663.400%</t>
+          <t>2663.400%</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
@@ -9644,7 +9644,7 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>2,022.700%</t>
+          <t>2022.700%</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
@@ -9739,7 +9739,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>2,090.700%</t>
+          <t>2090.700%</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>1,720.200%</t>
+          <t>1720.200%</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
@@ -9929,7 +9929,7 @@
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t>1,976.100%</t>
+          <t>1976.100%</t>
         </is>
       </c>
       <c r="L101" t="inlineStr">

</xml_diff>